<commit_message>
Update bigbasket_capstone.xlsx with new data revisions and enhanced analysis for better revenue insights.
</commit_message>
<xml_diff>
--- a/bigbasket_capstone.xlsx
+++ b/bigbasket_capstone.xlsx
@@ -6,17 +6,18 @@
     <sheet state="visible" name="Monthly Data" sheetId="1" r:id="rId5"/>
     <sheet state="visible" name="Pivot Table" sheetId="2" r:id="rId6"/>
     <sheet state="visible" name="Category Targets" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="Category Summary" sheetId="4" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId8"/>
+    <pivotCache cacheId="0" r:id="rId9"/>
   </pivotCaches>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="24">
   <si>
     <t>category</t>
   </si>
@@ -72,6 +73,15 @@
     <t>Household Essentials</t>
   </si>
   <si>
+    <t>variance</t>
+  </si>
+  <si>
+    <t>percentage_variance</t>
+  </si>
+  <si>
+    <t>tag</t>
+  </si>
+  <si>
     <t>SUM of total_revenue</t>
   </si>
   <si>
@@ -112,11 +122,14 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -134,6 +147,10 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -3284,4 +3301,200 @@
   <pageSetup orientation="landscape"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="19.0"/>
+    <col customWidth="1" min="2" max="2" width="13.14"/>
+    <col customWidth="1" min="3" max="3" width="17.57"/>
+    <col customWidth="1" min="4" max="4" width="8.29"/>
+    <col customWidth="1" min="5" max="5" width="18.86"/>
+    <col customWidth="1" min="6" max="6" width="19.57"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="str">
+        <f>'Pivot Table'!A2</f>
+        <v>Bakery</v>
+      </c>
+      <c r="B2" s="1">
+        <f>'Pivot Table'!B2</f>
+        <v>15410</v>
+      </c>
+      <c r="C2" s="1">
+        <f t="array" ref="C2">_xlfn.XLOOKUP(A2, 'Category Targets'!A:A, 'Category Targets'!B:B, "Not Found")</f>
+        <v>12000</v>
+      </c>
+      <c r="D2" s="1">
+        <f t="shared" ref="D2:D7" si="1">C2-B2</f>
+        <v>-3410</v>
+      </c>
+      <c r="E2" s="1">
+        <f t="shared" ref="E2:E7" si="2">((B2-C2)/C2)*100</f>
+        <v>28.41666667</v>
+      </c>
+      <c r="F2" s="1" t="str">
+        <f t="shared" ref="F2:F7" si="3">IF(B2&gt;=C2,"Above Target",IF(((C2-B2)/C2)*100&lt;=15,"Below Target - Watch","Below Target - Critical"))</f>
+        <v>Above Target</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="str">
+        <f>'Pivot Table'!A3</f>
+        <v>Dairy &amp; Eggs</v>
+      </c>
+      <c r="B3" s="1">
+        <f>'Pivot Table'!B3</f>
+        <v>14090</v>
+      </c>
+      <c r="C3" s="1">
+        <f t="array" ref="C3">_xlfn.XLOOKUP(A3, 'Category Targets'!A:A, 'Category Targets'!B:B, "Not Found")</f>
+        <v>16500</v>
+      </c>
+      <c r="D3" s="1">
+        <f t="shared" si="1"/>
+        <v>2410</v>
+      </c>
+      <c r="E3" s="1">
+        <f t="shared" si="2"/>
+        <v>-14.60606061</v>
+      </c>
+      <c r="F3" s="1" t="str">
+        <f t="shared" si="3"/>
+        <v>Below Target - Watch</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="str">
+        <f>'Pivot Table'!A4</f>
+        <v>Fruits &amp; Vegetables</v>
+      </c>
+      <c r="B4" s="1">
+        <f>'Pivot Table'!B4</f>
+        <v>9790</v>
+      </c>
+      <c r="C4" s="1">
+        <f t="array" ref="C4">_xlfn.XLOOKUP(A4, 'Category Targets'!A:A, 'Category Targets'!B:B, "Not Found")</f>
+        <v>12000</v>
+      </c>
+      <c r="D4" s="1">
+        <f t="shared" si="1"/>
+        <v>2210</v>
+      </c>
+      <c r="E4" s="1">
+        <f t="shared" si="2"/>
+        <v>-18.41666667</v>
+      </c>
+      <c r="F4" s="1" t="str">
+        <f t="shared" si="3"/>
+        <v>Below Target - Critical</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="str">
+        <f>'Pivot Table'!A5</f>
+        <v>Household Essentials</v>
+      </c>
+      <c r="B5" s="1">
+        <f>'Pivot Table'!B5</f>
+        <v>21715</v>
+      </c>
+      <c r="C5" s="1">
+        <f t="array" ref="C5">_xlfn.XLOOKUP(A5, 'Category Targets'!A:A, 'Category Targets'!B:B, "Not Found")</f>
+        <v>17000</v>
+      </c>
+      <c r="D5" s="1">
+        <f t="shared" si="1"/>
+        <v>-4715</v>
+      </c>
+      <c r="E5" s="1">
+        <f t="shared" si="2"/>
+        <v>27.73529412</v>
+      </c>
+      <c r="F5" s="1" t="str">
+        <f t="shared" si="3"/>
+        <v>Above Target</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="str">
+        <f>'Pivot Table'!A6</f>
+        <v>Personal Care</v>
+      </c>
+      <c r="B6" s="1">
+        <f>'Pivot Table'!B6</f>
+        <v>16382</v>
+      </c>
+      <c r="C6" s="1">
+        <f t="array" ref="C6">_xlfn.XLOOKUP(A6, 'Category Targets'!A:A, 'Category Targets'!B:B, "Not Found")</f>
+        <v>15500</v>
+      </c>
+      <c r="D6" s="1">
+        <f t="shared" si="1"/>
+        <v>-882</v>
+      </c>
+      <c r="E6" s="1">
+        <f t="shared" si="2"/>
+        <v>5.690322581</v>
+      </c>
+      <c r="F6" s="1" t="str">
+        <f t="shared" si="3"/>
+        <v>Above Target</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="str">
+        <f>'Pivot Table'!A7</f>
+        <v>Snacks &amp; Beverages</v>
+      </c>
+      <c r="B7" s="1">
+        <f>'Pivot Table'!B7</f>
+        <v>10895</v>
+      </c>
+      <c r="C7" s="1">
+        <f t="array" ref="C7">_xlfn.XLOOKUP(A7, 'Category Targets'!A:A, 'Category Targets'!B:B, "Not Found")</f>
+        <v>13000</v>
+      </c>
+      <c r="D7" s="1">
+        <f t="shared" si="1"/>
+        <v>2105</v>
+      </c>
+      <c r="E7" s="1">
+        <f t="shared" si="2"/>
+        <v>-16.19230769</v>
+      </c>
+      <c r="F7" s="1" t="str">
+        <f t="shared" si="3"/>
+        <v>Below Target - Critical</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update bigbasket_capstone.xlsx with further data revisions and refined analysis for enhanced revenue insights.
</commit_message>
<xml_diff>
--- a/bigbasket_capstone.xlsx
+++ b/bigbasket_capstone.xlsx
@@ -17,12 +17,21 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="26">
   <si>
     <t>category</t>
   </si>
   <si>
+    <t>target_revenue_inr</t>
+  </si>
+  <si>
+    <t>Fruits &amp; Vegetables</t>
+  </si>
+  <si>
     <t>month</t>
+  </si>
+  <si>
+    <t>Dairy &amp; Eggs</t>
   </si>
   <si>
     <t>order_count</t>
@@ -34,10 +43,19 @@
     <t>avg_revenue</t>
   </si>
   <si>
+    <t>Snacks &amp; Beverages</t>
+  </si>
+  <si>
     <t>Bakery</t>
   </si>
   <si>
+    <t>Personal Care</t>
+  </si>
+  <si>
     <t>2026-01</t>
+  </si>
+  <si>
+    <t>Household Essentials</t>
   </si>
   <si>
     <t>2026-02</t>
@@ -46,40 +64,28 @@
     <t>2026-03</t>
   </si>
   <si>
+    <t>variance</t>
+  </si>
+  <si>
+    <t>percentage_variance</t>
+  </si>
+  <si>
     <t>2026-04</t>
+  </si>
+  <si>
+    <t>tag</t>
+  </si>
+  <si>
+    <t>SQL Total (Part 1)</t>
+  </si>
+  <si>
+    <t>Matches Part 1 SQL total?</t>
   </si>
   <si>
     <t>2026-05</t>
   </si>
   <si>
     <t>2026-06</t>
-  </si>
-  <si>
-    <t>Dairy &amp; Eggs</t>
-  </si>
-  <si>
-    <t>target_revenue_inr</t>
-  </si>
-  <si>
-    <t>Fruits &amp; Vegetables</t>
-  </si>
-  <si>
-    <t>Snacks &amp; Beverages</t>
-  </si>
-  <si>
-    <t>Personal Care</t>
-  </si>
-  <si>
-    <t>Household Essentials</t>
-  </si>
-  <si>
-    <t>variance</t>
-  </si>
-  <si>
-    <t>percentage_variance</t>
-  </si>
-  <si>
-    <t>tag</t>
   </si>
   <si>
     <t>SUM of total_revenue</t>
@@ -95,7 +101,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -106,6 +112,10 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <color rgb="FFD1D5DA"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="2">
@@ -122,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -130,11 +140,55 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="4">
+    <dxf>
+      <font/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF6AA84F"/>
+          <bgColor rgb="FF6AA84F"/>
+        </patternFill>
+      </fill>
+      <border/>
+    </dxf>
+    <dxf>
+      <font/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB7E1CD"/>
+          <bgColor rgb="FFB7E1CD"/>
+        </patternFill>
+      </fill>
+      <border/>
+    </dxf>
+    <dxf>
+      <font/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <border/>
+    </dxf>
+    <dxf>
+      <font/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+      <border/>
+    </dxf>
+  </dxfs>
 </styleSheet>
 </file>
 
@@ -630,24 +684,24 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C2" s="1">
         <v>6.0</v>
@@ -661,10 +715,10 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C3" s="1">
         <v>8.0</v>
@@ -678,10 +732,10 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C4" s="1">
         <v>11.0</v>
@@ -695,10 +749,10 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C5" s="1">
         <v>13.0</v>
@@ -712,10 +766,10 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="C6" s="1">
         <v>15.0</v>
@@ -729,10 +783,10 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="C7" s="1">
         <v>14.0</v>
@@ -746,10 +800,10 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C8" s="1">
         <v>9.0</v>
@@ -763,10 +817,10 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C9" s="1">
         <v>8.0</v>
@@ -780,10 +834,10 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C10" s="1">
         <v>15.0</v>
@@ -797,10 +851,10 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C11" s="1">
         <v>9.0</v>
@@ -814,10 +868,10 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="C12" s="1">
         <v>14.0</v>
@@ -831,10 +885,10 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="C13" s="1">
         <v>11.0</v>
@@ -848,10 +902,10 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C14" s="1">
         <v>12.0</v>
@@ -865,10 +919,10 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C15" s="1">
         <v>13.0</v>
@@ -882,10 +936,10 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>8</v>
       </c>
       <c r="C16" s="1">
         <v>13.0</v>
@@ -899,10 +953,10 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C17" s="1">
         <v>14.0</v>
@@ -916,10 +970,10 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="C18" s="1">
         <v>12.0</v>
@@ -933,10 +987,10 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="C19" s="1">
         <v>9.0</v>
@@ -950,10 +1004,10 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C20" s="1">
         <v>10.0</v>
@@ -967,10 +1021,10 @@
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="1" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C21" s="1">
         <v>16.0</v>
@@ -984,10 +1038,10 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="1" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C22" s="1">
         <v>8.0</v>
@@ -1001,10 +1055,10 @@
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="C23" s="1">
         <v>17.0</v>
@@ -1018,10 +1072,10 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="1" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="C24" s="1">
         <v>16.0</v>
@@ -1035,10 +1089,10 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="1" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="C25" s="1">
         <v>12.0</v>
@@ -1052,10 +1106,10 @@
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="1" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C26" s="1">
         <v>12.0</v>
@@ -1069,10 +1123,10 @@
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="1" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C27" s="1">
         <v>8.0</v>
@@ -1086,10 +1140,10 @@
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="1" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C28" s="1">
         <v>11.0</v>
@@ -1103,10 +1157,10 @@
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="1" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C29" s="1">
         <v>9.0</v>
@@ -1120,10 +1174,10 @@
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="1" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="C30" s="1">
         <v>13.0</v>
@@ -1137,10 +1191,10 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="1" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="C31" s="1">
         <v>13.0</v>
@@ -1154,10 +1208,10 @@
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C32" s="1">
         <v>10.0</v>
@@ -1171,10 +1225,10 @@
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C33" s="1">
         <v>11.0</v>
@@ -1188,10 +1242,10 @@
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C34" s="1">
         <v>15.0</v>
@@ -1205,10 +1259,10 @@
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C35" s="1">
         <v>19.0</v>
@@ -1222,10 +1276,10 @@
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="C36" s="1">
         <v>13.0</v>
@@ -1239,10 +1293,10 @@
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="C37" s="1">
         <v>15.0</v>
@@ -2264,12 +2318,12 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="B2" s="1">
         <v>12000.0</v>
@@ -2277,7 +2331,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B3" s="1">
         <v>16500.0</v>
@@ -2285,7 +2339,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B4" s="1">
         <v>13000.0</v>
@@ -2293,7 +2347,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B5" s="1">
         <v>15500.0</v>
@@ -2301,7 +2355,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B6" s="1">
         <v>17000.0</v>
@@ -2309,7 +2363,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B7" s="1">
         <v>12000.0</v>
@@ -3316,6 +3370,8 @@
     <col customWidth="1" min="4" max="4" width="8.29"/>
     <col customWidth="1" min="5" max="5" width="18.86"/>
     <col customWidth="1" min="6" max="6" width="19.57"/>
+    <col customWidth="1" min="7" max="7" width="15.71"/>
+    <col customWidth="1" min="8" max="8" width="23.0"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3323,18 +3379,24 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3363,6 +3425,13 @@
         <f t="shared" ref="F2:F7" si="3">IF(B2&gt;=C2,"Above Target",IF(((C2-B2)/C2)*100&lt;=15,"Below Target - Watch","Below Target - Critical"))</f>
         <v>Above Target</v>
       </c>
+      <c r="G2" s="2">
+        <v>15410.0</v>
+      </c>
+      <c r="H2" s="1" t="str">
+        <f t="shared" ref="H2:H7" si="4">IF(B2=G2,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="str">
@@ -3389,6 +3458,13 @@
         <f t="shared" si="3"/>
         <v>Below Target - Watch</v>
       </c>
+      <c r="G3" s="2">
+        <v>14090.0</v>
+      </c>
+      <c r="H3" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>Yes</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="str">
@@ -3415,6 +3491,13 @@
         <f t="shared" si="3"/>
         <v>Below Target - Critical</v>
       </c>
+      <c r="G4" s="2">
+        <v>9790.0</v>
+      </c>
+      <c r="H4" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>Yes</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="str">
@@ -3441,6 +3524,13 @@
         <f t="shared" si="3"/>
         <v>Above Target</v>
       </c>
+      <c r="G5" s="2">
+        <v>21715.0</v>
+      </c>
+      <c r="H5" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>Yes</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="str">
@@ -3467,6 +3557,13 @@
         <f t="shared" si="3"/>
         <v>Above Target</v>
       </c>
+      <c r="G6" s="2">
+        <v>16382.0</v>
+      </c>
+      <c r="H6" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>Yes</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="str">
@@ -3493,8 +3590,38 @@
         <f t="shared" si="3"/>
         <v>Below Target - Critical</v>
       </c>
+      <c r="G7" s="2">
+        <v>10895.0</v>
+      </c>
+      <c r="H7" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="E11" s="3"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="F2:F7">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>F2="Above Target"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H10">
+    <cfRule type="notContainsBlanks" dxfId="1" priority="2">
+      <formula>LEN(TRIM(H10))&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F7">
+    <cfRule type="expression" dxfId="2" priority="3">
+      <formula>F2="Below Target - Watch"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F7">
+    <cfRule type="expression" dxfId="3" priority="4">
+      <formula>F2="Below Target - Critical"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>